<commit_message>
fix(documents): 위임장(heyman) 위임받는자 법인등록번호 교정 120111-0922270→110111-7526176
위임장 4.위임장!C25(위임받는 자=주식회사 헤이맨) 법인등록번호가 잘못된 값이라
heyman 실제 법인등록번호(통관 등록증/말소증과 동일)로 교정.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/resources/templates/heyman/power_of_attorney.xlsx
+++ b/resources/templates/heyman/power_of_attorney.xlsx
@@ -161,7 +161,7 @@
   </si>
   <si>
     <r>
-      <t xml:space="preserve">120111-0922270</t>
+      <t xml:space="preserve">110111-7526176</t>
     </r>
   </si>
   <si>
@@ -1261,7 +1261,7 @@
       <c r="C25" s="25" t="inlineStr">
         <is>
           <r>
-            <t xml:space="preserve">120111-0922270</t>
+            <t xml:space="preserve">110111-7526176</t>
           </r>
         </is>
       </c>

</xml_diff>